<commit_message>
Populate Complete Care facility list (92 locations) in wound volume workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CgSWz6arLBfkX8CeobngWG
</commit_message>
<xml_diff>
--- a/deliverables/Complete_Care_Wound_Volumes_TEMPLATE.xlsx
+++ b/deliverables/Complete_Care_Wound_Volumes_TEMPLATE.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -470,48 +470,51 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>To fill: once credits are restored, for each Complete Care SOC ID run</t>
-        </is>
-      </c>
-    </row>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Facility list populated: 92 locations from mycompletecare.com/locations (fetched 2026-10-07). SOC IDs and volumes still blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  get_account_clinical_practice(breakdown='by_code', codeType='hcpcs', codes=[HCPCS list])</t>
+          <t>To fill: once credits are restored, for each Complete Care SOC ID run</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  get_account_clinical_practice(breakdown='by_code', codeType='icdcm', codes=[ICD list])</t>
+          <t xml:space="preserve">  get_account_clinical_practice(breakdown='by_code', codeType='hcpcs', codes=[HCPCS list])</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t xml:space="preserve">  get_account_clinical_practice(breakdown='by_code', codeType='icdcm', codes=[ICD list])</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>and enter results on 'Volumes (long)'. 'Facility x Code' is a matrix of the same data.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Code list: see 'Code List'. Q-codes are a subset of high-volume skin substitutes; extend as needed.</t>
-        </is>
-      </c>
-    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>Code list: see 'Code List'. Q-codes are a subset of high-volume skin substitutes; extend as needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Debridement (11042-11047, 97597/8) is grouped with conservative care as standard-of-care; separate if the owner defines conservative care more narrowly.</t>
         </is>
@@ -1516,7 +1519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1568,6 +1571,2505 @@
       <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Complete Care at Annapolis</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>900 Van Buren St, Annapolis, MD 21403</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Annapolis</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Phone (410) 267-8653. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Complete Care at Arbors</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1750 NJ-37, Toms River, NJ 08757</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Toms River</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Phone (732) 914-0090. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Complete Care at Barn Hill</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>249 High St, Newton, NJ 07860</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Newton</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Phone (973) 383-5600. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Complete Care at Bayshore</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>715 N Beers St, Holmdel, NJ 07733</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Holmdel</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Phone (732) 847-3000. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Complete Care at Berkshire</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>5501 Perkiomen Ave, Reading, PA 19606</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Phone (610) 779-0600. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Complete Care at Bey Lea</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1351 Old Freehold Rd, Toms River, NJ 08753</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Toms River</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Phone (732) 240-0090. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Complete Care at Bey Lea Assisted Living</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1351 Old Freehold Rd, Toms River, NJ 08753</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Toms River</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Assisted living / residential (per name)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Phone (732) 240-0090. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Complete Care at Brackenville</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>100 St Claire Dr, Hockessin, DE 19707</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Hockessin</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Phone (302) 234-5420. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Complete Care at Brakeley Park</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>290 Red School Ln, Phillipsburg, NJ 08865</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Phillipsburg</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Phone (908) 859-2800. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Complete Care at Brick</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>415 Jack Martin Blvd, Brick Township, NJ 08724</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Brick Township</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Phone (732) 206-8000. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Complete Care at Burlington Woods</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>115 Sunset Rd, Burlington, NJ 08016</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Burlington</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Phone (609) 387-3620. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Complete Care at Care Age</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1755 N Barker Rd, Brookfield, WI 53045</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Brookfield</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Phone (262) 821-3939. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Complete Care at Cedar Grove</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>536 Ridge Rd, Cedar Grove, NJ 07009</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Cedar Grove</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Phone (973) 239-9300. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Complete Care at Chestnut Hill</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>360 Chestnut St, Passaic, NJ 07055</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Passaic</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Phone (973) 777-7800. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Chestnut Hill Residences by Complete Care</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>338 Chestnut St, Passaic, NJ 07055</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Passaic</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Assisted living / residential (per name)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Phone (973) 777-7800. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Complete Care at Christian Home</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>452 Fox Lake Rd, Waupun, WI 53963</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Waupun</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Phone (920) 324-9051. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Complete Care at Clark</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1213 Westfield Ave, Clark, NJ 07066</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Clark</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Phone (732) 396-7100. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Complete Care at Corsica Hills</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>205 Armstrong St, Centreville, MD 21617</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Centreville</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Phone (410) 758-2323. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Complete Care at Court House</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>144 Magnolia Dr, Middle Township, NJ 08210</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Middle Township</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Phone (609) 465-7171. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Complete Care at Dawnview</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1 Diane Dr, Fort Ashby, WV 26719</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Fort Ashby</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>WV</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Phone (304) 298-3602. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Complete Care at Fair Lawn Edge</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>77 E 43rd St, Paterson, NJ 07514</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Paterson</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Phone (973) 754-6700. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Complete Care at Fox Hill</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1253 Hartford Turnpike, Vernon, CT 06066</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Vernon</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Phone (860) 875-0771. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Complete Care at Germantown</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>10915 Bernies Way, Germantown, WI 53022</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Germantown</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Phone (262) 509-3300. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Complete Care at Glendale</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>4 Hazel Ave, Naugatuck, CT 06770</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Naugatuck</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Phone (203) 723-1456. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Complete Care at Glendale West</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>6263 N Green Bay Ave, Glendale, WI 53209</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Glendale</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Phone (414) 351-0543. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Complete Care at Grande Prairie</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>10330 Prairie Ridge Blvd, Pleasant Prairie, WI 53158</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Pleasant Prairie</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Phone (262) 612-2800. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Complete Care at Green Acres</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1931 Lakewood Rd, Toms River, NJ 08755</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Toms River</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Phone (732) 286-2323. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Complete Care at Green Knoll</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>875 US-202, Bridgewater, NJ 08807</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Bridgewater</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Phone (908) 526-8600. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Complete Care at Groton Regency</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1145 Poquonnock Rd, Groton, CT 06340</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Groton</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Phone (860) 446-9960. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Complete Care at Groton Regency Residential Care Home</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1145 Poquonnock Rd, Groton, CT 06340</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Groton</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Assisted living / residential (per name)</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Phone (860) 446-9960. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Complete Care at Hagerstown</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>14014 Marsh Pike, Hagerstown, MD 21742</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Hagerstown</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Phone (301) 733-8700. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Complete Care at Hales Corners</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>9449 W Forest Home Ave, Hales Corners, WI 53130</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Hales Corners</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Phone (414) 529-6888. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Complete Care at Hamilton Plaza</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>56 Hamilton Ave, Passaic, NJ 07055</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Passaic</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Phone (973) 773-7070. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Complete Care at Harborage</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>7600 River Rd, North Bergen, NJ 07047</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>North Bergen</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Phone (201) 854-5400. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Complete Care at Harrington Court</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>59 Harrington Ct, Colchester, CT 06415</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Colchester</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Phone (860) 537-2339. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Complete Care at Harston Hall</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>350 Haws Ln, Flourtown, PA 19031</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Flourtown</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Phone (215) 836-3200. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Complete Care at Heritage</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>7232 German Hill Rd, Baltimore, MD 21222</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Baltimore</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Phone (410) 282-6310. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Complete Care at Hillside</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>810 S Broom St, Wilmington, DE 19805</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Wilmington</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Phone (302) 652-1181. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Complete Care at Holiday City</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>4 Plaza Dr, Toms River, NJ 08757</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Toms River</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Phone (732) 240-0900. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Complete Care at Holmdel</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>713 N Beers St, Holmdel, NJ 07733</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Holmdel</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Phone (732) 335-4405. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Complete Care at Hyattsville</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>4922 Lasalle Rd, Hyattsville, MD 20782</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Hyattsville</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Phone (301) 864-2333. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Complete Care at Inglemoor</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>333 Grand Ave, Englewood, NJ 07631</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Englewood</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Phone (201) 568-0900. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Complete Care at Jefferson Meadows</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1414 Jefferson St, Baraboo, WI 53913</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Baraboo</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Phone (608) 356-4838. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Complete Care at Kensington</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1810 Kensington Dr, Waukesha, WI 53188</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Waukesha</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Phone (262) 548-1400. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Complete Care at Kimberly Hall North</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1 Emerson Dr, Windsor, CT 06095</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Windsor</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Phone (860) 688-6443. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Complete Care at Kimberly Hall South</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1 Emerson Dr, Windsor, CT 06095</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Windsor</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Phone (860) 688-6443. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Complete Care at Kresson View</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2601 E Evesham Rd, Voorhees Township, NJ 08043</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Voorhees Township</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Phone (856) 596-1113. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Complete Care at La Plata</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1 Magnolia Dr, La Plata, MD 20646</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>La Plata</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Phone (301) 934-4001. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Complete Care at Laurelton</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>475 Jack Martin Blvd, Brick Township, NJ 08724</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Brick Township</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Phone (732) 458-6600. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Complete Care at Lehigh</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1718 Spring Creek Rd, Macungie, PA 18062</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Macungie</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Phone (610) 366-0500. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Complete Care at Madison</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>625 NJ-34, Matawan, NJ 07747</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Matawan</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Phone (732) 566-6400. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Complete Care at Manitowoc</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2021 S Alverno Rd, Manitowoc, WI 54220</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Manitowoc</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Phone (920) 683-4100. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Complete Care at Maple Grove</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>3401 Maple Grove Dr, Madison, WI 53719</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Madison</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Phone (608) 845-1000. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Complete Care at Marcella</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2305 Rancocas Rd, Burlington, NJ 08016</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Burlington</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Phone (609) 387-9300. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Complete Care at Margate Park</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>4920 N Kenmore Ave, Chicago, IL 60640</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Phone (773) 769-2700. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Complete Care at Mercerville</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2240 Whitehorse Mercerville Rd, Hamilton Township, NJ 08619</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Hamilton Township</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Phone (609) 586-7500. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Complete Care at Meriden</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>845 Paddock Ave, Meriden, CT 06450</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Meriden</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Phone (203) 238-2645. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Complete Care at Middlebury</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>778 Middlebury Rd, Middlebury, CT 06762</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Middlebury</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Phone (203) 758-2471. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Complete Care at Milford Manor</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>69 Maple Rd, West Milford, NJ 07480</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>West Milford</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Phone (973) 697-5640. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Complete Care at Monmouth</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>229 Bath Ave, Long Branch, NJ 07740</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Long Branch</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Phone (732) 229-4300. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Complete Care at Multi Medical Center</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>7700 York Rd, Towson, MD 21204</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Towson</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Phone (410) 821-5500. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Complete Care at Nazareth</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>814 Jackson St, Stoughton, WI 53589</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Stoughton</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Phone (608) 873-6448. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Complete Care at Oak Ridge</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1000 Association Dr, Charleston, WV 25311</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Charleston</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>WV</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Phone (304) 347-4372. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Complete Care at Ocean Grove</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>160 S Main St, Neptune Township, NJ 07756</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Neptune Township</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Phone (732) 481-8300. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Complete Care at Orange Park</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>140 Park Ave, East Orange, NJ 07017</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>East Orange</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Phone (973) 677-1500. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Complete Care at Park Place</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2 Deerpark Dr, South Brunswick Township, NJ 08852</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>South Brunswick Township</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Phone (732) 274-1122. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Complete Care at Phillipsburg</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>843 Wilbur Ave, Phillipsburg, NJ 08865</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Phillipsburg</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Phone (908) 454-2627. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Complete Care at Plainfield</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>1340 Park Ave, Plainfield, NJ 07060</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Plainfield</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Phone (908) 754-3100. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Complete Care at Prospect Heights</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>336 Prospect Ave, Hackensack, NJ 07601</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Hackensack</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Phone (201) 678-1800. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Complete Care at Regent</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>50 Polifly Rd, Hackensack, NJ 07601</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Hackensack</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Phone (201) 646-1166. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Complete Care at Ridgewood</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>3205 Wood Rd, Racine, WI 53406</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Racine</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Phone (262) 554-6440. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Roosevelt Care Centers Edison</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>118 Parsonage Rd, Edison, NJ 08837</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Edison</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Phone (732) 321-6800. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Roosevelt Care Centers Old Bridge</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>1133 Marlboro Rd, Old Bridge, NJ 08857</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Old Bridge</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Phone (732) 360-9830. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Complete Care at Severna Park</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>310 Genesis Way, Severna Park, MD 21146</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Severna Park</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Phone (410) 544-4220. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Complete Care at Sheridan Commons</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>4538 N Beacon St, Chicago, IL 60640</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Phone (773) 275-7200. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Complete Care at Shorrock Gardens</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>75 Old Toms River Rd, Brick Township, NJ 08723</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Brick Township</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Phone (732) 451-1000. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Complete Care at Shrewsbury</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>89 Ave at the Cmns, Shrewsbury, NJ 07702</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Shrewsbury</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Phone (732) 676-5800. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Complete Care at Silver Lake</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>1080 Silver Lake Blvd, Dover, DE 19904</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Dover</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Phone (302) 734-5990. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Complete Care at Southpointe</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>4500 W Loomis Rd, Greenfield, WI 53220</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Greenfield</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Phone (414) 325-5300. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Complete Care at Springbrook</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>12325 New Hampshire Ave, Silver Spring, MD 20904</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Silver Spring</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Phone (301) 622-4600. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Complete Care at St. Vincent's</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>315 E Lindsley Rd, Cedar Grove, NJ 07009</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Cedar Grove</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Phone (973) 663-0011. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Complete Care at Summit Ridge</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>20 Summit St, West Orange, NJ 07052</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>West Orange</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Phone (973) 736-2000. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Complete Care at the Boulevard</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>5905 W Washington Blvd, Chicago, IL 60644</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Phone (773) 261-7074. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Complete Care at Voorhees</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>3001 E Evesham Rd, Voorhees Township, NJ 08043</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Voorhees Township</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Phone (856) 751-1600. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Complete Care at Wall</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>1725 Meridian Trail, Wall Township, NJ 07719</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Wall Township</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Phone (732) 312-1800. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Complete Care at Wayne Hills Rehab and Respiratory Center</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>130 Terhune Dr, Wayne, NJ 07470</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Wayne</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Phone (973) 839-4500. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Complete Care at West Caldwell</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>165 Fairfield Ave, West Caldwell, NJ 07006</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>West Caldwell</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Phone (973) 226-1100. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Complete Care at Westfield</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>1515 Lamberts Mill Rd, Westfield, NJ 07090</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Westfield</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Phone (908) 233-9700. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Complete Care at Wheaton</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>4011 Randolph Rd, Silver Spring, MD 20902</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Silver Spring</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Phone (301) 933-2500. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Complete Care at Whispering Woods</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>62 James St, Edison, NJ 08820</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Edison</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Phone (732) 744-5541. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Complete Care at Willow Creek</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>1165 Easton Ave, Franklin Township, NJ 08873</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Franklin Township</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Phone (732) 246-4100. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Complete Care at Woodlands</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>1400 Woodland Ave, Plainfield, NJ 07060</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Plainfield</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Phone (908) 753-1113. Source: mycompletecare.com/locations. SOC ID not yet matched in AcuityMD.</t>
         </is>
       </c>
     </row>
@@ -1673,7 +4175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT2"/>
+  <dimension ref="A1:AT94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2178,6 +4680,1110 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Complete Care at Annapolis</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Complete Care at Arbors</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Complete Care at Barn Hill</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Complete Care at Bayshore</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Complete Care at Berkshire</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Complete Care at Bey Lea</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Complete Care at Bey Lea Assisted Living</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Complete Care at Brackenville</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Complete Care at Brakeley Park</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Complete Care at Brick</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Complete Care at Burlington Woods</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Complete Care at Care Age</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Complete Care at Cedar Grove</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Complete Care at Chestnut Hill</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Chestnut Hill Residences by Complete Care</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Complete Care at Christian Home</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Complete Care at Clark</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Complete Care at Corsica Hills</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Complete Care at Court House</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Complete Care at Dawnview</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>WV</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Complete Care at Fair Lawn Edge</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Complete Care at Fox Hill</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Complete Care at Germantown</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Complete Care at Glendale</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Complete Care at Glendale West</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Complete Care at Grande Prairie</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Complete Care at Green Acres</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Complete Care at Green Knoll</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Complete Care at Groton Regency</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Complete Care at Groton Regency Residential Care Home</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Complete Care at Hagerstown</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Complete Care at Hales Corners</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Complete Care at Hamilton Plaza</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Complete Care at Harborage</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Complete Care at Harrington Court</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Complete Care at Harston Hall</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Complete Care at Heritage</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Complete Care at Hillside</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Complete Care at Holiday City</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Complete Care at Holmdel</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Complete Care at Hyattsville</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Complete Care at Inglemoor</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Complete Care at Jefferson Meadows</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Complete Care at Kensington</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Complete Care at Kimberly Hall North</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Complete Care at Kimberly Hall South</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Complete Care at Kresson View</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Complete Care at La Plata</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Complete Care at Laurelton</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Complete Care at Lehigh</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Complete Care at Madison</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Complete Care at Manitowoc</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Complete Care at Maple Grove</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Complete Care at Marcella</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Complete Care at Margate Park</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Complete Care at Mercerville</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Complete Care at Meriden</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Complete Care at Middlebury</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Complete Care at Milford Manor</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Complete Care at Monmouth</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Complete Care at Multi Medical Center</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Complete Care at Nazareth</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Complete Care at Oak Ridge</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>WV</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Complete Care at Ocean Grove</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Complete Care at Orange Park</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Complete Care at Park Place</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Complete Care at Phillipsburg</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Complete Care at Plainfield</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Complete Care at Prospect Heights</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Complete Care at Regent</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Complete Care at Ridgewood</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Roosevelt Care Centers Edison</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Roosevelt Care Centers Old Bridge</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Complete Care at Severna Park</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Complete Care at Sheridan Commons</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Complete Care at Shorrock Gardens</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Complete Care at Shrewsbury</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Complete Care at Silver Lake</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Complete Care at Southpointe</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Complete Care at Springbrook</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Complete Care at St. Vincent's</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Complete Care at Summit Ridge</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Complete Care at the Boulevard</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Complete Care at Voorhees</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Complete Care at Wall</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Complete Care at Wayne Hills Rehab and Respiratory Center</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Complete Care at West Caldwell</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Complete Care at Westfield</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Complete Care at Wheaton</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Complete Care at Whispering Woods</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Complete Care at Willow Creek</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Complete Care at Woodlands</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>